<commit_message>
state: session end 2026-08-10T10:02Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN8"/>
+  <dimension ref="A1:AN9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1303,9 +1303,131 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2026-08-10T10:00:58.162Z</v>
+      </c>
+      <c r="B9">
+        <v>24583.8</v>
+      </c>
+      <c r="C9">
+        <v>24600</v>
+      </c>
+      <c r="D9">
+        <v>0.84</v>
+      </c>
+      <c r="E9">
+        <v>24500</v>
+      </c>
+      <c r="F9">
+        <v>24600</v>
+      </c>
+      <c r="G9">
+        <v>24000</v>
+      </c>
+      <c r="H9">
+        <v>24600</v>
+      </c>
+      <c r="I9">
+        <v>25000</v>
+      </c>
+      <c r="J9">
+        <v>24700</v>
+      </c>
+      <c r="K9">
+        <v>15</v>
+      </c>
+      <c r="L9">
+        <v>43</v>
+      </c>
+      <c r="M9">
+        <v>8602555</v>
+      </c>
+      <c r="N9">
+        <v>64724985</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Call Unwinding 9x/1811225 | Put Writing 6x/5321225 | Put Unwinding 5x/828490 | Call Covering 4x/2452840 | Call Writing 14x/29441035 | Put Buying 14x/33173985 | Put Covering 6x/298740</v>
+      </c>
+      <c r="P9">
+        <v>18.35</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R9">
+        <v>0.467</v>
+      </c>
+      <c r="S9">
+        <v>0.519</v>
+      </c>
+      <c r="T9">
+        <v>15.265</v>
+      </c>
+      <c r="U9">
+        <v>0.0005</v>
+      </c>
+      <c r="V9">
+        <v>1.525</v>
+      </c>
+      <c r="W9" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X9">
+        <v>83</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z9">
+        <v>100</v>
+      </c>
+      <c r="AA9" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AB9">
+        <v>30</v>
+      </c>
+      <c r="AC9" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AD9">
+        <v>25</v>
+      </c>
+      <c r="AE9">
+        <v>50000</v>
+      </c>
+      <c r="AF9" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG9" t="str">
+        <v>BUY 24600PE | SELL 24550PE</v>
+      </c>
+      <c r="AH9">
+        <v>7</v>
+      </c>
+      <c r="AI9">
+        <v>20.45</v>
+      </c>
+      <c r="AJ9">
+        <v>10.22</v>
+      </c>
+      <c r="AK9">
+        <v>40.9</v>
+      </c>
+      <c r="AL9">
+        <v>4652</v>
+      </c>
+      <c r="AM9">
+        <v>9305</v>
+      </c>
+      <c r="AN9">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-11T08:23Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -3,7 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="2026-08-10" sheetId="1" r:id="rId1"/>
+    <sheet name="Trades" sheetId="1" r:id="rId1"/>
+    <sheet name="2026-08-10" sheetId="2" r:id="rId2"/>
+    <sheet name="2026-08-11" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -397,6 +399,123 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>PosId</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Timestamp</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ExitTime</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Horizon</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Expiry</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Legs</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Lots</v>
+      </c>
+      <c r="I1" t="str">
+        <v>NetEntry</v>
+      </c>
+      <c r="J1" t="str">
+        <v>NetExit</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Result</v>
+      </c>
+      <c r="L1" t="str">
+        <v>ExitReason</v>
+      </c>
+      <c r="M1" t="str">
+        <v>PnL</v>
+      </c>
+      <c r="N1" t="str">
+        <v>RR</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Confidence</v>
+      </c>
+      <c r="P1" t="str">
+        <v>EntryBias</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>TrendAtEntry</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1786436512219</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-08-11T08:21:52.219Z</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>intraday</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-08-11</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="G2" t="str">
+        <v>BUY 24450PE | SELL 24400PE</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+      <c r="I2">
+        <v>15.6</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>OPEN</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2">
+        <v>2</v>
+      </c>
+      <c r="O2">
+        <v>83</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Flat</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AN9"/>
   <sheetData>
     <row r="1">
@@ -1430,4 +1549,259 @@
     <ignoredError numberStoredAsText="1" sqref="A1:AN9"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:AN2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Timestamp</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Spot</v>
+      </c>
+      <c r="C1" t="str">
+        <v>ATMStrike</v>
+      </c>
+      <c r="D1" t="str">
+        <v>PCR</v>
+      </c>
+      <c r="E1" t="str">
+        <v>S1</v>
+      </c>
+      <c r="F1" t="str">
+        <v>S2</v>
+      </c>
+      <c r="G1" t="str">
+        <v>S3</v>
+      </c>
+      <c r="H1" t="str">
+        <v>R1</v>
+      </c>
+      <c r="I1" t="str">
+        <v>R2</v>
+      </c>
+      <c r="J1" t="str">
+        <v>R3</v>
+      </c>
+      <c r="K1" t="str">
+        <v>BullishCount</v>
+      </c>
+      <c r="L1" t="str">
+        <v>BearishCount</v>
+      </c>
+      <c r="M1" t="str">
+        <v>BullishOI</v>
+      </c>
+      <c r="N1" t="str">
+        <v>BearishOI</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Buildup</v>
+      </c>
+      <c r="P1" t="str">
+        <v>AvgIV</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Bias</v>
+      </c>
+      <c r="R1" t="str">
+        <v>AvgCallDelta</v>
+      </c>
+      <c r="S1" t="str">
+        <v>AvgPutDelta</v>
+      </c>
+      <c r="T1" t="str">
+        <v>AvgTheta</v>
+      </c>
+      <c r="U1" t="str">
+        <v>AvgGamma</v>
+      </c>
+      <c r="V1" t="str">
+        <v>AvgVega</v>
+      </c>
+      <c r="W1" t="str">
+        <v>CandleTrend</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Confidence</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Strategy1</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>Strategy1Score</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>Strategy2</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>Strategy2Score</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>Strategy3</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>Strategy3Score</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>Capital</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>Strategy</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>Legs</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>Lots</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>EntryPrice</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>StopLoss</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>Target</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>Risk</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>Reward</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>RiskRewardRatio</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>2026-08-11T08:21:52.206Z</v>
+      </c>
+      <c r="B2">
+        <v>24460.1</v>
+      </c>
+      <c r="C2">
+        <v>24450</v>
+      </c>
+      <c r="D2">
+        <v>0.75</v>
+      </c>
+      <c r="E2">
+        <v>24400</v>
+      </c>
+      <c r="F2">
+        <v>24450</v>
+      </c>
+      <c r="G2">
+        <v>24500</v>
+      </c>
+      <c r="H2">
+        <v>24500</v>
+      </c>
+      <c r="I2">
+        <v>24600</v>
+      </c>
+      <c r="J2">
+        <v>24550</v>
+      </c>
+      <c r="K2">
+        <v>20</v>
+      </c>
+      <c r="L2">
+        <v>62</v>
+      </c>
+      <c r="M2">
+        <v>62758085</v>
+      </c>
+      <c r="N2">
+        <v>196554800</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Call Writing 29x/153921950 | Put Writing 17x/61084270 | Call Unwinding 12x/2743975 | Put Unwinding 3x/1673815 | Put Buying 13x/33093905 | Put Covering 8x/6794970</v>
+      </c>
+      <c r="P2">
+        <v>56.67</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R2">
+        <v>0.478</v>
+      </c>
+      <c r="S2">
+        <v>0.5</v>
+      </c>
+      <c r="T2">
+        <v>110.224</v>
+      </c>
+      <c r="U2">
+        <v>0.0006</v>
+      </c>
+      <c r="V2">
+        <v>0.252</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X2">
+        <v>83</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z2">
+        <v>100</v>
+      </c>
+      <c r="AA2" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AB2">
+        <v>40</v>
+      </c>
+      <c r="AC2" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AD2">
+        <v>25</v>
+      </c>
+      <c r="AE2">
+        <v>50000</v>
+      </c>
+      <c r="AF2" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG2" t="str">
+        <v>BUY 24450PE | SELL 24400PE</v>
+      </c>
+      <c r="AH2">
+        <v>1</v>
+      </c>
+      <c r="AI2">
+        <v>15.6</v>
+      </c>
+      <c r="AJ2">
+        <v>7.8</v>
+      </c>
+      <c r="AK2">
+        <v>31.2</v>
+      </c>
+      <c r="AL2">
+        <v>507</v>
+      </c>
+      <c r="AM2">
+        <v>1014</v>
+      </c>
+      <c r="AN2">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN2"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-11T08:52Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -1712,7 +1712,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN29"/>
+  <dimension ref="A1:AN31"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4940,9 +4940,253 @@
         <v>2</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>2026-08-11T08:51:20.243Z</v>
+      </c>
+      <c r="B30">
+        <v>24454.2</v>
+      </c>
+      <c r="C30">
+        <v>24450</v>
+      </c>
+      <c r="D30">
+        <v>0.77</v>
+      </c>
+      <c r="E30">
+        <v>24450</v>
+      </c>
+      <c r="F30">
+        <v>24400</v>
+      </c>
+      <c r="G30">
+        <v>24500</v>
+      </c>
+      <c r="H30">
+        <v>24500</v>
+      </c>
+      <c r="I30">
+        <v>24600</v>
+      </c>
+      <c r="J30">
+        <v>24550</v>
+      </c>
+      <c r="K30">
+        <v>27</v>
+      </c>
+      <c r="L30">
+        <v>21</v>
+      </c>
+      <c r="M30">
+        <v>121936620</v>
+      </c>
+      <c r="N30">
+        <v>90573080</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Put Buying 13x/83391815 | Call Unwinding 3x/393315 | Call Writing 3x/931125 | Call Covering 6x/2993315 | Call Buying 12x/115826490 | Put Unwinding 6x/3083405 | Put Covering 2x/5856825 | Put Writing 3x/33410</v>
+      </c>
+      <c r="P30">
+        <v>64.16</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>Range</v>
+      </c>
+      <c r="R30">
+        <v>0.471</v>
+      </c>
+      <c r="S30">
+        <v>0.504</v>
+      </c>
+      <c r="T30">
+        <v>164.842</v>
+      </c>
+      <c r="U30">
+        <v>0.0006</v>
+      </c>
+      <c r="V30">
+        <v>0.209</v>
+      </c>
+      <c r="W30" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X30">
+        <v>83</v>
+      </c>
+      <c r="Y30" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="Z30">
+        <v>70</v>
+      </c>
+      <c r="AA30" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AB30">
+        <v>50</v>
+      </c>
+      <c r="AC30" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AD30">
+        <v>50</v>
+      </c>
+      <c r="AE30">
+        <v>50000</v>
+      </c>
+      <c r="AF30" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AG30" t="str">
+        <v>SELL 24400PE | BUY 24350PE | SELL 24500CE | BUY 24550CE</v>
+      </c>
+      <c r="AH30">
+        <v>1</v>
+      </c>
+      <c r="AI30">
+        <v>-19.2</v>
+      </c>
+      <c r="AJ30">
+        <v>-28.8</v>
+      </c>
+      <c r="AK30">
+        <v>0</v>
+      </c>
+      <c r="AL30">
+        <v>624</v>
+      </c>
+      <c r="AM30">
+        <v>1248</v>
+      </c>
+      <c r="AN30">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>2026-08-11T08:52:20.449Z</v>
+      </c>
+      <c r="B31">
+        <v>24455.1</v>
+      </c>
+      <c r="C31">
+        <v>24450</v>
+      </c>
+      <c r="D31">
+        <v>0.78</v>
+      </c>
+      <c r="E31">
+        <v>24450</v>
+      </c>
+      <c r="F31">
+        <v>24400</v>
+      </c>
+      <c r="G31">
+        <v>24500</v>
+      </c>
+      <c r="H31">
+        <v>24500</v>
+      </c>
+      <c r="I31">
+        <v>24600</v>
+      </c>
+      <c r="J31">
+        <v>24550</v>
+      </c>
+      <c r="K31">
+        <v>18</v>
+      </c>
+      <c r="L31">
+        <v>34</v>
+      </c>
+      <c r="M31">
+        <v>42217240</v>
+      </c>
+      <c r="N31">
+        <v>153748855</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Put Writing 9x/39963170 | Put Unwinding 5x/2113995 | Call Writing 16x/128401910 | Call Covering 2x/20085 | Call Unwinding 7x/3372720 | Call Buying 2x/119990 | Put Buying 5x/13461305 | Put Covering 6x/8512920</v>
+      </c>
+      <c r="P31">
+        <v>63.81</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R31">
+        <v>0.47</v>
+      </c>
+      <c r="S31">
+        <v>0.504</v>
+      </c>
+      <c r="T31">
+        <v>169.214</v>
+      </c>
+      <c r="U31">
+        <v>0.0006</v>
+      </c>
+      <c r="V31">
+        <v>0.208</v>
+      </c>
+      <c r="W31" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X31">
+        <v>83</v>
+      </c>
+      <c r="Y31" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z31">
+        <v>100</v>
+      </c>
+      <c r="AA31" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AB31">
+        <v>40</v>
+      </c>
+      <c r="AC31" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AD31">
+        <v>25</v>
+      </c>
+      <c r="AE31">
+        <v>50000</v>
+      </c>
+      <c r="AF31" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG31" t="str">
+        <v>BUY 24450PE | SELL 24400PE</v>
+      </c>
+      <c r="AH31">
+        <v>1</v>
+      </c>
+      <c r="AI31">
+        <v>15.1</v>
+      </c>
+      <c r="AJ31">
+        <v>7.55</v>
+      </c>
+      <c r="AK31">
+        <v>30.2</v>
+      </c>
+      <c r="AL31">
+        <v>491</v>
+      </c>
+      <c r="AM31">
+        <v>981</v>
+      </c>
+      <c r="AN31">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-12T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -8059,7 +8059,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN66"/>
+  <dimension ref="A1:AN68"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -15417,9 +15417,205 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-08-12T07:00:42.777Z</v>
+      </c>
+      <c r="B67">
+        <v>24279.8</v>
+      </c>
+      <c r="C67">
+        <v>24300</v>
+      </c>
+      <c r="D67">
+        <v>0.66</v>
+      </c>
+      <c r="E67">
+        <v>24000</v>
+      </c>
+      <c r="F67">
+        <v>24300</v>
+      </c>
+      <c r="G67">
+        <v>23800</v>
+      </c>
+      <c r="H67">
+        <v>24500</v>
+      </c>
+      <c r="I67">
+        <v>24400</v>
+      </c>
+      <c r="J67">
+        <v>24600</v>
+      </c>
+      <c r="K67">
+        <v>55</v>
+      </c>
+      <c r="L67">
+        <v>12</v>
+      </c>
+      <c r="M67">
+        <v>80077400</v>
+      </c>
+      <c r="N67">
+        <v>20256210</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Put Writing 32x/28866175 | Call Buying 19x/51056785 | Put Unwinding 4x/154440 | Call Writing 11x/20081165 | Call Unwinding 1x/175045</v>
+      </c>
+      <c r="P67">
+        <v>10.78</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>Range</v>
+      </c>
+      <c r="R67">
+        <v>0.496</v>
+      </c>
+      <c r="S67">
+        <v>0.503</v>
+      </c>
+      <c r="T67">
+        <v>5.548</v>
+      </c>
+      <c r="U67">
+        <v>0.0005</v>
+      </c>
+      <c r="V67">
+        <v>5.644</v>
+      </c>
+      <c r="W67" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X67">
+        <v>50</v>
+      </c>
+      <c r="Y67" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="Z67">
+        <v>70</v>
+      </c>
+      <c r="AA67" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AB67">
+        <v>50</v>
+      </c>
+      <c r="AC67" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AD67">
+        <v>50</v>
+      </c>
+      <c r="AE67">
+        <v>50000</v>
+      </c>
+      <c r="AF67" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>2026-08-12T07:03:43.825Z</v>
+      </c>
+      <c r="B68">
+        <v>24285.65</v>
+      </c>
+      <c r="C68">
+        <v>24300</v>
+      </c>
+      <c r="D68">
+        <v>0.65</v>
+      </c>
+      <c r="E68">
+        <v>24000</v>
+      </c>
+      <c r="F68">
+        <v>24300</v>
+      </c>
+      <c r="G68">
+        <v>23800</v>
+      </c>
+      <c r="H68">
+        <v>24500</v>
+      </c>
+      <c r="I68">
+        <v>24400</v>
+      </c>
+      <c r="J68">
+        <v>24600</v>
+      </c>
+      <c r="K68">
+        <v>55</v>
+      </c>
+      <c r="L68">
+        <v>10</v>
+      </c>
+      <c r="M68">
+        <v>90078300</v>
+      </c>
+      <c r="N68">
+        <v>2684695</v>
+      </c>
+      <c r="O68" t="str">
+        <v>Put Writing 30x/28880020 | Call Buying 23x/61067825 | Call Unwinding 1x/325 | Call Writing 6x/2626715 | Put Unwinding 2x/130455 | Put Covering 2x/34190 | Put Buying 1x/23465</v>
+      </c>
+      <c r="P68">
+        <v>10.7</v>
+      </c>
+      <c r="Q68" t="str">
+        <v>Range</v>
+      </c>
+      <c r="R68">
+        <v>0.502</v>
+      </c>
+      <c r="S68">
+        <v>0.501</v>
+      </c>
+      <c r="T68">
+        <v>5.351</v>
+      </c>
+      <c r="U68">
+        <v>0.0005</v>
+      </c>
+      <c r="V68">
+        <v>5.562</v>
+      </c>
+      <c r="W68" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X68">
+        <v>50</v>
+      </c>
+      <c r="Y68" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="Z68">
+        <v>70</v>
+      </c>
+      <c r="AA68" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="AB68">
+        <v>50</v>
+      </c>
+      <c r="AC68" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AD68">
+        <v>50</v>
+      </c>
+      <c r="AE68">
+        <v>50000</v>
+      </c>
+      <c r="AF68" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN68"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-13T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -16365,7 +16365,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN66"/>
+  <dimension ref="A1:AN67"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -23387,9 +23387,107 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>2026-08-13T07:02:59.699Z</v>
+      </c>
+      <c r="B67">
+        <v>24394.85</v>
+      </c>
+      <c r="C67">
+        <v>24400</v>
+      </c>
+      <c r="D67">
+        <v>0.95</v>
+      </c>
+      <c r="E67">
+        <v>24400</v>
+      </c>
+      <c r="F67">
+        <v>24300</v>
+      </c>
+      <c r="G67">
+        <v>24000</v>
+      </c>
+      <c r="H67">
+        <v>24500</v>
+      </c>
+      <c r="I67">
+        <v>25000</v>
+      </c>
+      <c r="J67">
+        <v>24400</v>
+      </c>
+      <c r="K67">
+        <v>16</v>
+      </c>
+      <c r="L67">
+        <v>48</v>
+      </c>
+      <c r="M67">
+        <v>14040390</v>
+      </c>
+      <c r="N67">
+        <v>47063315</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Put Buying 18x/21604570 | Call Unwinding 5x/568425 | Call Buying 4x/15990 | Put Covering 4x/182000 | Call Covering 1x/48165 | Call Writing 21x/24708320 | Put Writing 7x/13945750 | Put Unwinding 4x/30485</v>
+      </c>
+      <c r="P67">
+        <v>10.86</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R67">
+        <v>0.486</v>
+      </c>
+      <c r="S67">
+        <v>0.498</v>
+      </c>
+      <c r="T67">
+        <v>5.301</v>
+      </c>
+      <c r="U67">
+        <v>0.0005</v>
+      </c>
+      <c r="V67">
+        <v>4.61</v>
+      </c>
+      <c r="W67" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X67">
+        <v>67</v>
+      </c>
+      <c r="Y67" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z67">
+        <v>100</v>
+      </c>
+      <c r="AA67" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AB67">
+        <v>70</v>
+      </c>
+      <c r="AC67" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AD67">
+        <v>30</v>
+      </c>
+      <c r="AE67">
+        <v>50000</v>
+      </c>
+      <c r="AF67" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN66"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN67"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-14T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -23690,7 +23690,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP61"/>
+  <dimension ref="A1:AP62"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -30570,9 +30570,137 @@
         <v/>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-08-14 12:33:07</v>
+      </c>
+      <c r="B62">
+        <v>24341.05</v>
+      </c>
+      <c r="C62">
+        <v>24350</v>
+      </c>
+      <c r="D62">
+        <v>0.84</v>
+      </c>
+      <c r="E62">
+        <v>24300</v>
+      </c>
+      <c r="F62">
+        <v>24350</v>
+      </c>
+      <c r="G62">
+        <v>24000</v>
+      </c>
+      <c r="H62">
+        <v>24500</v>
+      </c>
+      <c r="I62">
+        <v>24400</v>
+      </c>
+      <c r="J62">
+        <v>25000</v>
+      </c>
+      <c r="K62">
+        <v>6</v>
+      </c>
+      <c r="L62">
+        <v>55</v>
+      </c>
+      <c r="M62">
+        <v>3342690</v>
+      </c>
+      <c r="N62">
+        <v>99753810</v>
+      </c>
+      <c r="O62" t="str">
+        <v>Put Writing 6x/3342690 | Call Unwinding 5x/248040 | Call Writing 25x/55434015 | Put Buying 21x/44036980 | Put Covering 4x/34775</v>
+      </c>
+      <c r="P62">
+        <v>10.67</v>
+      </c>
+      <c r="Q62" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R62">
+        <v>0.495</v>
+      </c>
+      <c r="S62">
+        <v>0.497</v>
+      </c>
+      <c r="T62">
+        <v>4.451</v>
+      </c>
+      <c r="U62">
+        <v>0.0006</v>
+      </c>
+      <c r="V62">
+        <v>3.539</v>
+      </c>
+      <c r="W62" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X62">
+        <v>83</v>
+      </c>
+      <c r="Y62" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z62">
+        <v>100</v>
+      </c>
+      <c r="AA62" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AB62">
+        <v>75</v>
+      </c>
+      <c r="AC62" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AD62">
+        <v>70</v>
+      </c>
+      <c r="AE62">
+        <v>50000</v>
+      </c>
+      <c r="AF62" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AG62" t="str">
+        <v>BUY 24350PE | SELL 24300PE</v>
+      </c>
+      <c r="AH62">
+        <v>1</v>
+      </c>
+      <c r="AI62">
+        <v>20.45</v>
+      </c>
+      <c r="AJ62">
+        <v>10.22</v>
+      </c>
+      <c r="AK62" t="str">
+        <v>SIGNAL</v>
+      </c>
+      <c r="AL62">
+        <v>665</v>
+      </c>
+      <c r="AM62" t="str">
+        <v/>
+      </c>
+      <c r="AN62" t="str">
+        <v/>
+      </c>
+      <c r="AO62" t="str">
+        <v>ride</v>
+      </c>
+      <c r="AP62" t="str">
+        <v>same legs already traded today</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP62"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-17T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -36954,7 +36954,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP61"/>
+  <dimension ref="A1:AP63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -43924,9 +43924,205 @@
         <v>bias Bearish persisted 1/2 polls</v>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>2026-08-17 12:30:49</v>
+      </c>
+      <c r="B62">
+        <v>24288</v>
+      </c>
+      <c r="C62">
+        <v>24300</v>
+      </c>
+      <c r="D62">
+        <v>0.65</v>
+      </c>
+      <c r="E62">
+        <v>24300</v>
+      </c>
+      <c r="F62">
+        <v>24200</v>
+      </c>
+      <c r="G62">
+        <v>24250</v>
+      </c>
+      <c r="H62">
+        <v>24300</v>
+      </c>
+      <c r="I62">
+        <v>24400</v>
+      </c>
+      <c r="J62">
+        <v>24500</v>
+      </c>
+      <c r="K62">
+        <v>39</v>
+      </c>
+      <c r="L62">
+        <v>20</v>
+      </c>
+      <c r="M62">
+        <v>100299095</v>
+      </c>
+      <c r="N62">
+        <v>62233795</v>
+      </c>
+      <c r="O62" t="str">
+        <v>Call Covering 2x/16835 | Put Buying 3x/305500 | Call Buying 17x/55423615 | Put Covering 6x/753025 | Put Writing 12x/42729375 | Call Writing 11x/61175270 | Put Unwinding 8x/2129270</v>
+      </c>
+      <c r="P62">
+        <v>16.55</v>
+      </c>
+      <c r="Q62" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R62">
+        <v>0.471</v>
+      </c>
+      <c r="S62">
+        <v>0.513</v>
+      </c>
+      <c r="T62">
+        <v>13.667</v>
+      </c>
+      <c r="U62">
+        <v>0.0006</v>
+      </c>
+      <c r="V62">
+        <v>1.522</v>
+      </c>
+      <c r="W62" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X62">
+        <v>67</v>
+      </c>
+      <c r="Y62" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="Z62">
+        <v>75</v>
+      </c>
+      <c r="AA62" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AB62">
+        <v>50</v>
+      </c>
+      <c r="AC62" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AD62">
+        <v>30</v>
+      </c>
+      <c r="AE62">
+        <v>50000</v>
+      </c>
+      <c r="AF62" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-08-17 12:33:49</v>
+      </c>
+      <c r="B63">
+        <v>24293.9</v>
+      </c>
+      <c r="C63">
+        <v>24300</v>
+      </c>
+      <c r="D63">
+        <v>0.66</v>
+      </c>
+      <c r="E63">
+        <v>24300</v>
+      </c>
+      <c r="F63">
+        <v>24250</v>
+      </c>
+      <c r="G63">
+        <v>24200</v>
+      </c>
+      <c r="H63">
+        <v>24300</v>
+      </c>
+      <c r="I63">
+        <v>24400</v>
+      </c>
+      <c r="J63">
+        <v>24500</v>
+      </c>
+      <c r="K63">
+        <v>49</v>
+      </c>
+      <c r="L63">
+        <v>12</v>
+      </c>
+      <c r="M63">
+        <v>148120895</v>
+      </c>
+      <c r="N63">
+        <v>7594275</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Call Covering 2x/4550 | Put Buying 6x/2925130 | Put Writing 11x/41375360 | Call Unwinding 1x/17875 | Put Unwinding 13x/2829125 | Call Buying 23x/103911860 | Put Covering 1x/92690 | Call Writing 4x/4558580</v>
+      </c>
+      <c r="P63">
+        <v>17.23</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R63">
+        <v>0.478</v>
+      </c>
+      <c r="S63">
+        <v>0.508</v>
+      </c>
+      <c r="T63">
+        <v>13.404</v>
+      </c>
+      <c r="U63">
+        <v>0.0006</v>
+      </c>
+      <c r="V63">
+        <v>1.521</v>
+      </c>
+      <c r="W63" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X63">
+        <v>67</v>
+      </c>
+      <c r="Y63" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="Z63">
+        <v>75</v>
+      </c>
+      <c r="AA63" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AB63">
+        <v>60</v>
+      </c>
+      <c r="AC63" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="AD63">
+        <v>50</v>
+      </c>
+      <c r="AE63">
+        <v>50000</v>
+      </c>
+      <c r="AF63" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP63"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
state: session end 2026-08-20T10:04Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -2362,7 +2362,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP115"/>
+  <dimension ref="A1:AP116"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -13694,9 +13694,107 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>2026-08-20 15:30:56</v>
+      </c>
+      <c r="B116">
+        <v>24231.85</v>
+      </c>
+      <c r="C116">
+        <v>24250</v>
+      </c>
+      <c r="D116">
+        <v>0.65</v>
+      </c>
+      <c r="E116">
+        <v>24150</v>
+      </c>
+      <c r="F116">
+        <v>24100</v>
+      </c>
+      <c r="G116">
+        <v>24200</v>
+      </c>
+      <c r="H116">
+        <v>24200</v>
+      </c>
+      <c r="I116">
+        <v>24250</v>
+      </c>
+      <c r="J116">
+        <v>24300</v>
+      </c>
+      <c r="K116">
+        <v>0</v>
+      </c>
+      <c r="L116">
+        <v>2</v>
+      </c>
+      <c r="M116">
+        <v>0</v>
+      </c>
+      <c r="N116">
+        <v>163670</v>
+      </c>
+      <c r="O116" t="str">
+        <v>Call Unwinding 1x/163345 | Put Covering 1x/325</v>
+      </c>
+      <c r="P116">
+        <v>192.74</v>
+      </c>
+      <c r="Q116" t="str">
+        <v>Bearish</v>
+      </c>
+      <c r="R116">
+        <v>0.464</v>
+      </c>
+      <c r="S116">
+        <v>0.54</v>
+      </c>
+      <c r="T116">
+        <v>2808.103</v>
+      </c>
+      <c r="U116">
+        <v>0.0004</v>
+      </c>
+      <c r="V116">
+        <v>0</v>
+      </c>
+      <c r="W116" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X116">
+        <v>67</v>
+      </c>
+      <c r="Y116" t="str">
+        <v>Bear Put Spread</v>
+      </c>
+      <c r="Z116">
+        <v>100</v>
+      </c>
+      <c r="AA116" t="str">
+        <v>Buy Put</v>
+      </c>
+      <c r="AB116">
+        <v>60</v>
+      </c>
+      <c r="AC116" t="str">
+        <v>Iron Condor</v>
+      </c>
+      <c r="AD116">
+        <v>40</v>
+      </c>
+      <c r="AE116">
+        <v>50000</v>
+      </c>
+      <c r="AF116" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP115"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP116"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
state: session end 2026-08-21T07:05Z
</commit_message>
<xml_diff>
--- a/option_dashboard.xlsx
+++ b/option_dashboard.xlsx
@@ -13926,7 +13926,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AP62"/>
+  <dimension ref="A1:AP63"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -20484,9 +20484,107 @@
         <v>NO TRADE</v>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>2026-08-21 12:32:40</v>
+      </c>
+      <c r="B63">
+        <v>24244.3</v>
+      </c>
+      <c r="C63">
+        <v>24250</v>
+      </c>
+      <c r="D63">
+        <v>1.05</v>
+      </c>
+      <c r="E63">
+        <v>24200</v>
+      </c>
+      <c r="F63">
+        <v>24000</v>
+      </c>
+      <c r="G63">
+        <v>24300</v>
+      </c>
+      <c r="H63">
+        <v>24300</v>
+      </c>
+      <c r="I63">
+        <v>24500</v>
+      </c>
+      <c r="J63">
+        <v>24200</v>
+      </c>
+      <c r="K63">
+        <v>48</v>
+      </c>
+      <c r="L63">
+        <v>7</v>
+      </c>
+      <c r="M63">
+        <v>105257880</v>
+      </c>
+      <c r="N63">
+        <v>3160430</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Put Writing 23x/55025750 | Put Buying 2x/224640 | Call Covering 4x/25090 | Call Buying 18x/50097905 | Put Unwinding 3x/109135 | Put Covering 1x/1690 | Call Writing 4x/2934100</v>
+      </c>
+      <c r="P63">
+        <v>9.81</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>Bullish</v>
+      </c>
+      <c r="R63">
+        <v>0.515</v>
+      </c>
+      <c r="S63">
+        <v>0.486</v>
+      </c>
+      <c r="T63">
+        <v>3.619</v>
+      </c>
+      <c r="U63">
+        <v>0.0006</v>
+      </c>
+      <c r="V63">
+        <v>3.262</v>
+      </c>
+      <c r="W63" t="str">
+        <v>Flat</v>
+      </c>
+      <c r="X63">
+        <v>50</v>
+      </c>
+      <c r="Y63" t="str">
+        <v>Bull Call Spread</v>
+      </c>
+      <c r="Z63">
+        <v>100</v>
+      </c>
+      <c r="AA63" t="str">
+        <v>Long Straddle</v>
+      </c>
+      <c r="AB63">
+        <v>70</v>
+      </c>
+      <c r="AC63" t="str">
+        <v>Buy Call</v>
+      </c>
+      <c r="AD63">
+        <v>60</v>
+      </c>
+      <c r="AE63">
+        <v>50000</v>
+      </c>
+      <c r="AF63" t="str">
+        <v>NO TRADE</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AP62"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AP63"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>